<commit_message>
updated with failed scenario handling
</commit_message>
<xml_diff>
--- a/testData/Book1.xlsx
+++ b/testData/Book1.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BDDRealtimeProject\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A50716-BEEE-4676-B10A-63D57A1F6A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{64C24D4D-946A-4257-AAF9-AE41C656BE4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A466B15D-CE77-4E64-ACCA-0B2323982C74}"/>
   </bookViews>
   <sheets>
-    <sheet name="contactUs" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>